<commit_message>
cigna global script without nationality
</commit_message>
<xml_diff>
--- a/Input/Cigna_Global_Health/benefits.xlsx
+++ b/Input/Cigna_Global_Health/benefits.xlsx
@@ -1035,7 +1035,7 @@
         <v>$0, 20% Co-insurance, $5,000 Out of pocket</v>
       </c>
       <c r="AN6" s="1" t="str">
-        <v>$1,000, 0% Co-insurance</v>
+        <v>$150, 0% Co-insurance</v>
       </c>
       <c r="AT6" s="1" t="str">
         <v>Dental_Waiting_Period</v>
@@ -1046,7 +1046,7 @@
         <v>$0, 30% Co-insurance, $2,000 Out of pocket</v>
       </c>
       <c r="AN7" s="1" t="str">
-        <v>$1,000, 10% Co-insurance, $3,000 Out of pocket</v>
+        <v>$150, 10% Co-insurance, $3,000 Out of pocket</v>
       </c>
       <c r="AT7" s="1" t="str">
         <v>Emergency-Evacuation</v>
@@ -1057,186 +1057,186 @@
         <v>$0, 30% Co-insurance, $5,000 Out of pocket</v>
       </c>
       <c r="AN8" s="1" t="str">
-        <v>$1,000, 20% Co-insurance, $3,000 Out of pocket</v>
+        <v>$150, 20% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="9">
       <c r="AM9" s="1" t="str">
-        <v>$1,500, 0% Co-insurance, $0 Out of pocket</v>
+        <v>$375, 0% Co-insurance, $0 Out of pocket</v>
       </c>
       <c r="AN9" s="1" t="str">
-        <v>$1,000, 30% Co-insurance, $3,000 Out of pocket</v>
+        <v>$150, 30% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="10">
       <c r="AM10" s="1" t="str">
-        <v>$1,500, 10% Co-insurance, $2,000 Out of pocket</v>
+        <v>$375, 10% Co-insurance, $2,000 Out of pocket</v>
       </c>
       <c r="AN10" s="1" t="str">
-        <v>$1,500, 0% Co-insurance</v>
+        <v>$500, 0% Co-insurance</v>
       </c>
     </row>
     <row r="11">
       <c r="AM11" s="1" t="str">
-        <v>$1,500, 10% Co-insurance, $5,000 Out of pocket</v>
+        <v>$375, 10% Co-insurance, $5,000 Out of pocket</v>
       </c>
       <c r="AN11" s="1" t="str">
-        <v>$1,500, 10% Co-insurance, $3,000 Out of pocket</v>
+        <v>$500, 10% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="12">
       <c r="AM12" s="1" t="str">
-        <v>$1,500, 20% Co-insurance, $2,000 Out of pocket</v>
+        <v>$375, 20% Co-insurance, $2,000 Out of pocket</v>
       </c>
       <c r="AN12" s="1" t="str">
-        <v>$1,500, 20% Co-insurance, $3,000 Out of pocket</v>
+        <v>$500, 20% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="13">
       <c r="AM13" s="1" t="str">
-        <v>$1,500, 20% Co-insurance, $5,000 Out of pocket</v>
+        <v>$375, 20% Co-insurance, $5,000 Out of pocket</v>
       </c>
       <c r="AN13" s="1" t="str">
-        <v>$1,500, 30% Co-insurance, $3,000 Out of pocket</v>
+        <v>$500, 30% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="14">
       <c r="AM14" s="1" t="str">
-        <v>$1,500, 30% Co-insurance, $2,000 Out of pocket</v>
+        <v>$375, 30% Co-insurance, $2,000 Out of pocket</v>
       </c>
       <c r="AN14" s="1" t="str">
-        <v>$150, 0% Co-insurance</v>
+        <v>$1,000, 0% Co-insurance</v>
       </c>
     </row>
     <row r="15">
       <c r="AM15" s="1" t="str">
-        <v>$1,500, 30% Co-insurance, $5,000 Out of pocket</v>
+        <v>$375, 30% Co-insurance, $5,000 Out of pocket</v>
       </c>
       <c r="AN15" s="1" t="str">
-        <v>$150, 10% Co-insurance, $3,000 Out of pocket</v>
+        <v>$1,000, 10% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="16">
       <c r="AM16" s="1" t="str">
-        <v>$10,000, 0% Co-insurance, $0 Out of pocket</v>
+        <v>$750, 0% Co-insurance, $0 Out of pocket</v>
       </c>
       <c r="AN16" s="1" t="str">
-        <v>$150, 20% Co-insurance, $3,000 Out of pocket</v>
+        <v>$1,000, 20% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="17">
       <c r="AM17" s="1" t="str">
-        <v>$10,000, 10% Co-insurance, $2,000 Out of pocket</v>
+        <v>$750, 10% Co-insurance, $2,000 Out of pocket</v>
       </c>
       <c r="AN17" s="1" t="str">
-        <v>$150, 30% Co-insurance, $3,000 Out of pocket</v>
+        <v>$1,000, 30% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="18">
       <c r="AM18" s="1" t="str">
-        <v>$10,000, 10% Co-insurance, $5,000 Out of pocket</v>
+        <v>$750, 10% Co-insurance, $5,000 Out of pocket</v>
       </c>
       <c r="AN18" s="1" t="str">
-        <v>$500, 0% Co-insurance</v>
+        <v>$1,500, 0% Co-insurance</v>
       </c>
     </row>
     <row r="19">
       <c r="AM19" s="1" t="str">
-        <v>$10,000, 20% Co-insurance, $2,000 Out of pocket</v>
+        <v>$750, 20% Co-insurance, $2,000 Out of pocket</v>
       </c>
       <c r="AN19" s="1" t="str">
-        <v>$500, 10% Co-insurance, $3,000 Out of pocket</v>
+        <v>$1,500, 10% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="20">
       <c r="AM20" s="1" t="str">
-        <v>$10,000, 20% Co-insurance, $5,000 Out of pocket</v>
+        <v>$750, 20% Co-insurance, $5,000 Out of pocket</v>
       </c>
       <c r="AN20" s="1" t="str">
-        <v>$500, 20% Co-insurance, $3,000 Out of pocket</v>
+        <v>$1,500, 20% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="21">
       <c r="AM21" s="1" t="str">
-        <v>$10,000, 30% Co-insurance, $2,000 Out of pocket</v>
+        <v>$750, 30% Co-insurance, $2,000 Out of pocket</v>
       </c>
       <c r="AN21" s="1" t="str">
-        <v>$500, 30% Co-insurance, $3,000 Out of pocket</v>
+        <v>$1,500, 30% Co-insurance, $3,000 Out of pocket</v>
       </c>
     </row>
     <row r="22">
       <c r="AM22" s="1" t="str">
-        <v>$10,000, 30% Co-insurance, $5,000 Out of pocket</v>
+        <v>$750, 30% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="23">
       <c r="AM23" s="1" t="str">
-        <v>$3,000, 0% Co-insurance, $0 Out of pocket</v>
+        <v>$1,500, 0% Co-insurance, $0 Out of pocket</v>
       </c>
     </row>
     <row r="24">
       <c r="AM24" s="1" t="str">
-        <v>$3,000, 10% Co-insurance, $2,000 Out of pocket</v>
+        <v>$1,500, 10% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="25">
       <c r="AM25" s="1" t="str">
-        <v>$3,000, 10% Co-insurance, $5,000 Out of pocket</v>
+        <v>$1,500, 10% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="26">
       <c r="AM26" s="1" t="str">
-        <v>$3,000, 20% Co-insurance, $2,000 Out of pocket</v>
+        <v>$1,500, 20% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="27">
       <c r="AM27" s="1" t="str">
-        <v>$3,000, 20% Co-insurance, $5,000 Out of pocket</v>
+        <v>$1,500, 20% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="28">
       <c r="AM28" s="1" t="str">
-        <v>$3,000, 30% Co-insurance, $2,000 Out of pocket</v>
+        <v>$1,500, 30% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="29">
       <c r="AM29" s="1" t="str">
-        <v>$3,000, 30% Co-insurance, $5,000 Out of pocket</v>
+        <v>$1,500, 30% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="30">
       <c r="AM30" s="1" t="str">
-        <v>$375, 0% Co-insurance, $0 Out of pocket</v>
+        <v>$3,000, 0% Co-insurance, $0 Out of pocket</v>
       </c>
     </row>
     <row r="31">
       <c r="AM31" s="1" t="str">
-        <v>$375, 10% Co-insurance, $2,000 Out of pocket</v>
+        <v>$3,000, 10% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="32">
       <c r="AM32" s="1" t="str">
-        <v>$375, 10% Co-insurance, $5,000 Out of pocket</v>
+        <v>$3,000, 10% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="33">
       <c r="AM33" s="1" t="str">
-        <v>$375, 20% Co-insurance, $2,000 Out of pocket</v>
+        <v>$3,000, 20% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="34">
       <c r="AM34" s="1" t="str">
-        <v>$375, 20% Co-insurance, $5,000 Out of pocket</v>
+        <v>$3,000, 20% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="35">
       <c r="AM35" s="1" t="str">
-        <v>$375, 30% Co-insurance, $2,000 Out of pocket</v>
+        <v>$3,000, 30% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="36">
       <c r="AM36" s="1" t="str">
-        <v>$375, 30% Co-insurance, $5,000 Out of pocket</v>
+        <v>$3,000, 30% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="37">
@@ -1276,37 +1276,37 @@
     </row>
     <row r="44">
       <c r="AM44" s="1" t="str">
-        <v>$750, 0% Co-insurance, $0 Out of pocket</v>
+        <v>$10,000, 0% Co-insurance, $0 Out of pocket</v>
       </c>
     </row>
     <row r="45">
       <c r="AM45" s="1" t="str">
-        <v>$750, 10% Co-insurance, $2,000 Out of pocket</v>
+        <v>$10,000, 10% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="46">
       <c r="AM46" s="1" t="str">
-        <v>$750, 10% Co-insurance, $5,000 Out of pocket</v>
+        <v>$10,000, 10% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="47">
       <c r="AM47" s="1" t="str">
-        <v>$750, 20% Co-insurance, $2,000 Out of pocket</v>
+        <v>$10,000, 20% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="48">
       <c r="AM48" s="1" t="str">
-        <v>$750, 20% Co-insurance, $5,000 Out of pocket</v>
+        <v>$10,000, 20% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
     <row r="49">
       <c r="AM49" s="1" t="str">
-        <v>$750, 30% Co-insurance, $2,000 Out of pocket</v>
+        <v>$10,000, 30% Co-insurance, $2,000 Out of pocket</v>
       </c>
     </row>
     <row r="50">
       <c r="AM50" s="1" t="str">
-        <v>$750, 30% Co-insurance, $5,000 Out of pocket</v>
+        <v>$10,000, 30% Co-insurance, $5,000 Out of pocket</v>
       </c>
     </row>
   </sheetData>

</xml_diff>